<commit_message>
Support embedded product photos in Excel import and refresh template.
- Extract images anchored over rows via exceljs, upload to Supabase
  Storage (bucket `product-images`, auto-created public), merge URLs.
- New template: styled headers, frozen row, currency/gender dropdowns,
  instruction sheet, sample row without price (skipped on import).
- Bot help and stats now mention embedded photos and show upload count.
- Env knobs: EXCEL_IMPORT_MAX_IMAGES_PER_PRODUCT (8), MAX_IMAGE_BYTES (4MB).
</commit_message>
<xml_diff>
--- a/docs/excel-import-template.xlsx
+++ b/docs/excel-import-template.xlsx
@@ -5,13 +5,45 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Товары" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Инструкция" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <t>Обязательно. Уникальный код товара.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <r>
+          <t>Обязательно. Число. Валюта — в соседней колонке.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <r>
+          <t>Вставьте фото поверх ячеек этой колонки (Вставка → Рисунки → Поместить над ячейками) или впишите ссылки через пробел.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>Артикул</t>
   </si>
@@ -40,59 +72,89 @@
     <t>Пол</t>
   </si>
   <si>
-    <t>AB-1001</t>
-  </si>
-  <si>
-    <t>Кроссовки беговые</t>
-  </si>
-  <si>
-    <t>Nike</t>
+    <t>ОБРАЗЕЦ</t>
+  </si>
+  <si>
+    <t>Пример товара (эту строку можно удалить — она не импортируется, т.к. без цены)</t>
   </si>
   <si>
     <t>Кроссовки</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>CNY</t>
   </si>
   <si>
     <t>40,41,42,43</t>
   </si>
   <si>
-    <t>https://example.com/img/ab1001-1.jpg https://example.com/img/ab1001-2.jpg</t>
+    <t>Вставьте фото в эту строку или впишите ссылки через пробел</t>
   </si>
   <si>
     <t>мужской</t>
   </si>
   <si>
-    <t>AB-1002</t>
-  </si>
-  <si>
-    <t>Очки солнцезащитные</t>
-  </si>
-  <si>
-    <t>Gucci</t>
-  </si>
-  <si>
-    <t>Очки</t>
-  </si>
-  <si>
-    <t>RUB</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>https://example.com/img/ab1002.jpg</t>
-  </si>
-  <si>
-    <t>женский</t>
+    <t>ИНСТРУКЦИЯ ПО ЗАПОЛНЕНИЮ ТАБЛИЦЫ</t>
+  </si>
+  <si>
+    <t>1. Одна строка листа «Товары» = один товар.</t>
+  </si>
+  <si>
+    <t>2. Обязательные колонки: АРТИКУЛ и ЦЕНА. Без них товар не добавится.</t>
+  </si>
+  <si>
+    <t>3. Артикул — уникальный код товара. Если товар с таким артикулом уже есть в магазине, он обновится.</t>
+  </si>
+  <si>
+    <t>4. Цена — число. Валюта: CNY (юани, цена пересчитается с наценкой) или RUB (рубли, итоговая розничная цена).</t>
+  </si>
+  <si>
+    <t>5. Размеры — в одной ячейке через запятую, например: 40,41,42,43. Для одежды: S,M,L,XL.</t>
+  </si>
+  <si>
+    <t>6. Пол — мужской / женский / unisex (или оставьте пустым).</t>
+  </si>
+  <si>
+    <t>7. Категория — например: Кроссовки, Очки, Одежда. Новая категория создастся автоматически.</t>
+  </si>
+  <si>
+    <t>ФОТОГРАФИИ — два способа:</t>
+  </si>
+  <si>
+    <t>• Вставить картинкой: «Вставка → Рисунки → Поместить НАД ячейками» и расположить фото</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  напротив строки своего товара (в колонке «Фото»). До 8 фото на товар.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Важно: НЕ используйте вариант «Поместить В ячейку» — такие фото не распознаются.</t>
+  </si>
+  <si>
+    <t>• Или ссылками: вписать в колонку «Фото» адреса картинок через пробел или запятую.</t>
+  </si>
+  <si>
+    <t>ЛИМИТЫ ФАЙЛА: не более 8 МБ и не более 2000 товаров в одном файле.</t>
+  </si>
+  <si>
+    <t>Готовый файл отправьте в Telegram-бот (чат админ-бота, просто пришлите файл .xlsx).</t>
+  </si>
+  <si>
+    <t>Бот пришлёт отчёт: сколько товаров создано, обновлено и пропущено.</t>
+  </si>
+  <si>
+    <t>Первую строку (заголовки колонок) не удалять и не переименовывать!</t>
+  </si>
+  <si>
+    <t>Строку-образец можно удалить или перезаписать своим товаром.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -102,17 +164,37 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF808080"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5496"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -120,13 +202,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -466,97 +569,1212 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I1000"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="9" width="20" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E2">
-        <v>450</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="257" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="258" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="259" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="260" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="261" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="262" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="263" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="264" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="265" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="266" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="267" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="268" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="269" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="270" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="271" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="272" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="273" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="274" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="275" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="276" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="277" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="278" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="279" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="280" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="281" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="282" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="283" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="284" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="285" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="286" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="287" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="288" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="289" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="290" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="291" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="292" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="293" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="294" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="295" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="296" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="297" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="298" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="299" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="300" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="301" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="302" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="303" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="304" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="305" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="306" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="307" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="308" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="309" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="310" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="311" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="312" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="313" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="314" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="315" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="316" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="317" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="318" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="319" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="320" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="321" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="322" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="323" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="324" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="325" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="326" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="327" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="328" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="329" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="330" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="331" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="332" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="333" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="334" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="335" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="336" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="337" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="338" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="339" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="340" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="341" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="342" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="343" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="344" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="345" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="346" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="347" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="348" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="349" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="350" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="351" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="352" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="353" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="354" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="355" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="356" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="357" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="358" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="359" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="360" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="361" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="362" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="363" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="364" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="365" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="366" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="367" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="368" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="369" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="370" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="371" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="372" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="373" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="374" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="375" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="376" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="377" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="378" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="379" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="380" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="381" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="382" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="383" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="384" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="385" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="386" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="387" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="388" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="389" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="390" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="391" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="392" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="393" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="394" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="395" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="396" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="397" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="398" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="399" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="400" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="401" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="402" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="403" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="404" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="405" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="406" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="407" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="408" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="409" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="410" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="411" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="412" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="413" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="414" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="415" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="416" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="417" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="418" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="419" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="420" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="421" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="422" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="423" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="424" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="425" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="426" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="427" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="428" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="429" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="430" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="431" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="432" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="433" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="434" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="435" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="436" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="437" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="438" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="439" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="440" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="441" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="442" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="443" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="444" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="445" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="446" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="447" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="448" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="449" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="450" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="451" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="452" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="453" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="454" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="455" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="456" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="457" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="458" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="459" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="460" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="461" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="462" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="463" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="464" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="465" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="466" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="467" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="468" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="469" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="470" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="471" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="472" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="473" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="474" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="475" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="476" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="477" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="478" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="479" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="480" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="481" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="482" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="483" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="484" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="485" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="486" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="487" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="488" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="489" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="490" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="491" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="492" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="493" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="494" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="495" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="496" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="497" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="498" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="499" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="500" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="501" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="502" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="503" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="504" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="505" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="506" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="507" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="508" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="509" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="510" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="511" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="512" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="513" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="514" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="515" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="516" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="517" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="518" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="519" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="520" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="521" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="522" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="523" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="524" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="525" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="526" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="527" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="528" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="529" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="530" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="531" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="532" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="533" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="534" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="535" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="536" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="537" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="538" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="539" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="540" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="541" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="542" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="543" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="544" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="545" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="546" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="547" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="548" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="549" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="550" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="551" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="552" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="553" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="554" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="555" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="556" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="557" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="558" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="559" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="560" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="561" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="562" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="563" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="564" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="565" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="566" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="567" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="568" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="569" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="570" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="571" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="572" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="573" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="574" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="575" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="576" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="577" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="578" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="579" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="580" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="581" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="582" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="583" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="584" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="585" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="586" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="587" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="588" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="589" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="590" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="591" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="592" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="593" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="594" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="595" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="596" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="597" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="598" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="599" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="600" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="601" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="602" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="603" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="604" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="605" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="606" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="607" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="608" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="609" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="610" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="611" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="612" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="613" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="614" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="615" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="616" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="617" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="618" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="619" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="620" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="621" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="622" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="623" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="624" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="625" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="626" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="627" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="628" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="629" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="630" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="631" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="632" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="633" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="634" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="635" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="636" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="637" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="638" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="639" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="640" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="641" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="642" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="643" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="644" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="645" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="646" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="647" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="648" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="649" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="650" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="651" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="652" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="653" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="654" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="655" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="656" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="657" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="658" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="659" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="660" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="661" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="662" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="663" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="664" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="665" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="666" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="667" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="668" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="669" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="670" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="671" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="672" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="673" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="674" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="675" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="676" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="677" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="678" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="679" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="680" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="681" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="682" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="683" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="684" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="685" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="686" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="687" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="688" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="689" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="690" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="691" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="692" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="693" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="694" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="695" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="696" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="697" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="698" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="699" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="700" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="701" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="702" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="703" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="704" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="705" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="706" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="707" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="708" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="709" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="710" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="711" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="712" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="713" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="714" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="715" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="716" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="717" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="718" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="719" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="720" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="721" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="722" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="723" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="724" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="725" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="726" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="727" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="728" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="729" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="730" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="731" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="732" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="733" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="734" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="735" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="736" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="737" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="738" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="739" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="740" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="741" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="742" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="743" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="744" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="745" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="746" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="747" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="748" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="749" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="750" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="751" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="752" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="753" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="754" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="755" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="756" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="757" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="758" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="759" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="760" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="761" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="762" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="763" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="764" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="765" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="766" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="767" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="768" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="769" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="770" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="771" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="772" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="773" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="774" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="775" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="776" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="777" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="778" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="779" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="780" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="781" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="782" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="783" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="784" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="785" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="786" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="787" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="788" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="789" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="790" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="791" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="792" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="793" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="794" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="795" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="796" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="797" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="798" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="799" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="800" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="801" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="802" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="803" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="804" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="805" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="806" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="807" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="808" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="809" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="810" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="811" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="812" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="813" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="814" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="815" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="816" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="817" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="818" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="819" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="820" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="821" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="822" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="823" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="824" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="825" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="826" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="827" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="828" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="829" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="830" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="831" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="832" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="833" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="834" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="835" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="836" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="837" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="838" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="839" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="840" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="841" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="842" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="843" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="844" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="845" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="846" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="847" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="848" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="849" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="850" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="851" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="852" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="853" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="854" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="855" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="856" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="857" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="858" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="859" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="860" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="861" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="862" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="863" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="864" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="865" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="866" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="867" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="868" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="869" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="870" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="871" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="872" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="873" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="874" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="875" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="876" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="877" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="878" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="879" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="880" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="881" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="882" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="883" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="884" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="885" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="886" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="887" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="888" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="889" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="890" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="891" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="892" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="893" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="894" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="895" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="896" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="897" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="898" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="899" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="900" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="901" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="902" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="903" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="904" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="905" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="906" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="907" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="908" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="909" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="910" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="911" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="912" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="913" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="914" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="915" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="916" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="917" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="918" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="919" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="920" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="921" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="922" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="923" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="924" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="925" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="926" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="927" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="928" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="929" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="930" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="931" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="932" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="933" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="934" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="935" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="936" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="937" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="938" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="939" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="940" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="941" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="942" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="943" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="944" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="945" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="946" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="947" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="948" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="949" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="950" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="951" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="952" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="953" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="954" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="955" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="956" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="957" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="958" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="959" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="960" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="961" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="962" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="963" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="964" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="965" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="966" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="967" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="968" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="969" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="970" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="971" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="972" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="973" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="974" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="975" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="976" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="977" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="978" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="979" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="980" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="981" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="982" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="983" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="984" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="985" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="986" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="987" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="988" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="989" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="990" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="991" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="992" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="993" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="994" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="995" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="996" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="997" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="998" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="999" spans="6:9" x14ac:dyDescent="0.25"/>
+    <row r="1000" spans="6:9" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="F10:F1000">
+      <formula1>"CNY,RUB"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F2:F1000">
+      <formula1>"CNY,RUB"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I10:I1000">
+      <formula1>"мужской,женский,unisex"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I1000">
+      <formula1>"мужской,женский,unisex"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A22"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="110" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E3">
-        <v>12500</v>
-      </c>
-      <c r="F3" t="s">
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="s">
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H3" t="s">
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make Excel template universal and auto-fit columns.
- Sizes column now covers shoes (40,41,42), clothing (S,M,L,XL),
  glasses (52-18-140), and accessories (one size / empty).
- Auto-fit column widths based on cell content (like VBA AutoFit).
- Min column widths set as floor, expanded as needed.
</commit_message>
<xml_diff>
--- a/docs/excel-import-template.xlsx
+++ b/docs/excel-import-template.xlsx
@@ -31,6 +31,13 @@
         </r>
       </text>
     </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <t>Через запятую. Для обуви: 40,41,42. Для одежды: S,M,L,XL. Для очков: 52-18-140. Для аксессуаров: один размер или пустое.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="H1" authorId="0">
       <text>
         <r>
@@ -43,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
   <si>
     <t>Артикул</t>
   </si>
@@ -111,7 +118,19 @@
     <t>4. Цена — число. Валюта: CNY (юани, цена пересчитается с наценкой) или RUB (рубли, итоговая розничная цена).</t>
   </si>
   <si>
-    <t>5. Размеры — в одной ячейке через запятую, например: 40,41,42,43. Для одежды: S,M,L,XL.</t>
+    <t>5. Размеры — в одной ячейке через запятую. Формат зависит от категории товара:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Кроссовки/обувь: 40,41,42,43 (европейские размеры)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Одежда: S,M,L,XL или 44,46,48,50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Очки: 52-18-140 (линза-мост-дужка) или один размер</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Аксессуары: один размер, универсальный или оставьте пустым</t>
   </si>
   <si>
     <t>6. Пол — мужской / женский / unisex (или оставьте пустым).</t>
@@ -572,14 +591,14 @@
   <dimension ref="A1:I1000"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="60" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1661,7 +1680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1714,27 +1733,27 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
@@ -1744,22 +1763,22 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
@@ -1769,12 +1788,32 @@
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make sizes column truly universal for any product category.
- Instruction now covers: shoes, clothing, glasses, electronics
  (memory/color), jewelry (ring size/chain length), watches (diameter),
  accessories, and any custom parameters.
- Column note clarified: "any variants/parameters via comma".
- Template regenerated.
</commit_message>
<xml_diff>
--- a/docs/excel-import-template.xlsx
+++ b/docs/excel-import-template.xlsx
@@ -34,7 +34,7 @@
     <comment ref="G1" authorId="0">
       <text>
         <r>
-          <t>Через запятую. Для обуви: 40,41,42. Для одежды: S,M,L,XL. Для очков: 52-18-140. Для аксессуаров: один размер или пустое.</t>
+          <t>Любые варианты/параметры товара через запятую: размеры (40,41,42), память (64GB,128GB), цвет (Black,White), длина (40cm,45cm) и т.д. Можно оставить пустым.</t>
         </r>
       </text>
     </comment>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
   <si>
     <t>Артикул</t>
   </si>
@@ -118,10 +118,10 @@
     <t>4. Цена — число. Валюта: CNY (юани, цена пересчитается с наценкой) или RUB (рубли, итоговая розничная цена).</t>
   </si>
   <si>
-    <t>5. Размеры — в одной ячейке через запятую. Формат зависит от категории товара:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   • Кроссовки/обувь: 40,41,42,43 (европейские размеры)</t>
+    <t>5. Размеры/Параметры — в одной ячейке через запятую. Сюда вписываются ЛЮБЫЕ варианты или характеристики товара:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Обувь: 40,41,42,43 (европейские размеры)</t>
   </si>
   <si>
     <t xml:space="preserve">   • Одежда: S,M,L,XL или 44,46,48,50</t>
@@ -130,13 +130,25 @@
     <t xml:space="preserve">   • Очки: 52-18-140 (линза-мост-дужка) или один размер</t>
   </si>
   <si>
+    <t xml:space="preserve">   • Техника: 64GB,128GB,256GB (память) или Black,White,Blue (цвет)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Ювелирка: 16,17,18 (размер кольца) или 40cm,45cm,50cm (длина цепочки)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Часы: 38mm,40mm,42mm (диаметр корпуса)</t>
+  </si>
+  <si>
     <t xml:space="preserve">   • Аксессуары: один размер, универсальный или оставьте пустым</t>
   </si>
   <si>
+    <t xml:space="preserve">   Если у товара нет вариантов — оставьте пустым или впишите одну характеристику.</t>
+  </si>
+  <si>
     <t>6. Пол — мужской / женский / unisex (или оставьте пустым).</t>
   </si>
   <si>
-    <t>7. Категория — например: Кроссовки, Очки, Одежда. Новая категория создастся автоматически.</t>
+    <t>7. Категория — например: Кроссовки, Очки, Одежда, Техника, Ювелирка. Новая категория создастся автоматически.</t>
   </si>
   <si>
     <t>ФОТОГРАФИИ — два способа:</t>
@@ -1680,7 +1692,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -1753,27 +1765,27 @@
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
@@ -1783,22 +1795,22 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
@@ -1808,12 +1820,32 @@
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>